<commit_message>
Planning 12/10-1/11 refait : Jennyfer en fermeture, dimanches Yassine + Sara + Rose/Jennyfer en alternance
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017sABE5Ku13TMCaT7NQhVkc
</commit_message>
<xml_diff>
--- a/Planning_12oct-1nov.xlsx
+++ b/Planning_12oct-1nov.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="77">
   <si>
     <t xml:space="preserve">CEDIF Saint-Antoine — Planning du lundi 12 octobre au dimanche 1er novembre 2026</t>
   </si>
@@ -91,90 +91,108 @@
     <t xml:space="preserve">RETOUR SÉMINAIRE (trajet)</t>
   </si>
   <si>
-    <t xml:space="preserve">14:00-19:40</t>
+    <t xml:space="preserve">15:00-17:40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11:50-15:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16:00-19:40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jeudi 15/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15:00-18:50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12:00-15:40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12:25-15:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vendredi 16/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INDISPONIBLE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Samedi 17/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15:00-19:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dimanche 18/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10:50-13:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14:00-19:10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14:05-19:10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10:50-14:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15:00-19:10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL SEMAINE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contrat 35h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contrat 25h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contrat 15h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SEMAINE 2 — du 19/10 au 25/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lundi 19/10</t>
   </si>
   <si>
     <t xml:space="preserve">15:00-17:50</t>
   </si>
   <si>
-    <t xml:space="preserve">Jeudi 15/10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15:00-18:50</t>
+    <t xml:space="preserve">Mardi 20/10</t>
   </si>
   <si>
     <t xml:space="preserve">11:40-15:00</t>
   </si>
   <si>
-    <t xml:space="preserve">16:00-19:40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vendredi 16/10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INDISPONIBLE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Samedi 17/10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10:10-15:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dimanche 18/10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10:50-14:00</t>
+    <t xml:space="preserve">Mercredi 21/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jeudi 22/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vendredi 23/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Samedi 24/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dimanche 25/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11:10-15:00</t>
   </si>
   <si>
     <t xml:space="preserve">16:00-19:10</t>
   </si>
   <si>
-    <t xml:space="preserve">TOTAL SEMAINE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contrat 35h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contrat 25h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contrat 15h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SEMAINE 2 — du 19/10 au 25/10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lundi 19/10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mardi 20/10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mercredi 21/10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jeudi 22/10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vendredi 23/10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11:00-13:20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Samedi 24/10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dimanche 25/10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11:10-15:00</t>
-  </si>
-  <si>
     <t xml:space="preserve">SEMAINE 3 — du 26/10 au 01/11</t>
   </si>
   <si>
@@ -190,15 +208,9 @@
     <t xml:space="preserve">Jeudi 29/10</t>
   </si>
   <si>
-    <t xml:space="preserve">11:50-15:00</t>
-  </si>
-  <si>
     <t xml:space="preserve">Vendredi 30/10</t>
   </si>
   <si>
-    <t xml:space="preserve">10:00-14:00</t>
-  </si>
-  <si>
     <t xml:space="preserve">Samedi 31/10</t>
   </si>
   <si>
@@ -217,25 +229,25 @@
     <t xml:space="preserve">NOTES</t>
   </si>
   <si>
-    <t xml:space="preserve">• Séminaire Yassine (lun 12 – mer 14) : heures de séminaire comptées (lun 3h30, mar 7h30 avec 1h de déjeuner). Temps de trajet à récupérer avant fin novembre (option 1 du mail).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Yassine indisponible le ven 16 : 27h cette semaine (séminaire 11h + magasin 16h).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Lun 12 et mar 13 : intérimaire 11:00-19:00 (pause 15-16h). Rose ouvre et ferme (elle a les clés) avec pause 14-15h couverte par l'intérimaire. Mardi, Rose passe la commande.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Livraisons jeu/ven : 3 personnes le ven 23 et le ven 30 ; seulement 2 les jeu 15, ven 16, jeu 22 et jeu 29 → renfort possible : intérim ou heures complémentaires de Jennyfer.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Sara indisponible sam 24 / dim 25 : Jennyfer fait le samedi, Yassine et Rose le dimanche.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Jennyfer en congé du sam 31/10 au lun 2/11 : remplacée par Rose le samedi 31 (5h40 de congé décomptées).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Dim 1er novembre (Toussaint) : magasin fermé → Sara ne fait que le samedi cette semaine-là (8h au lieu de 15h).</t>
+    <t xml:space="preserve">• Jennyfer est toujours en fermeture. Dimanche : Yassine + Sara + Rose ou Jennyfer en alternance (18/10 Jennyfer, 25/10 Rose, 1/11 Jennyfer mais fermé).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Séminaire Yassine (lun 12 – mer 14) : heures comptées (lun 3h30, mar 7h30 avec 1h de déjeuner). Temps de trajet à récupérer avant fin novembre (option 1 du mail). Yassine indisponible le ven 16.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Lun 12 et mar 13 : intérimaire 11:00-19:00 (pause 15-16h). Rose ouvre et ferme (clés), sa pause 14-15h est couverte par l'intérimaire. Mardi 13, Rose passe la commande.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Livraisons : 3 personnes le jeu 15 et le ven 30 ; 2 personnes les ven 16, jeu 22, ven 23 et jeu 29 → renfort possible (intérim / heures complémentaires).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Sara indisponible sam 24 / dim 25 : samedi Yassine + Jennyfer, dimanche Yassine + Rose (seulement 2 personnes).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Jennyfer en congé du sam 31/10 au lun 2/11 (6h15 décomptées le samedi) : Rose travaille le samedi 31.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Dim 1er novembre (Toussaint) : magasin fermé → Sara ne fait que le samedi cette semaine-là (8h).</t>
   </si>
   <si>
     <t xml:space="preserve">• Totaux journaliers saisis à la main (pause non comptée) ; les totaux semaine sont des formules.</t>
@@ -1025,21 +1037,23 @@
       </c>
       <c r="C9" s="12"/>
       <c r="D9" s="13"/>
-      <c r="E9" s="14"/>
+      <c r="E9" s="14" t="s">
+        <v>14</v>
+      </c>
       <c r="F9" s="14" t="s">
         <v>23</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.236111111111111</v>
+        <v>0.284722222222222</v>
       </c>
       <c r="H9" s="14" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="I9" s="14" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J9" s="13" t="n">
-        <v>0.291666666666667</v>
+        <v>0.284722222222222</v>
       </c>
       <c r="K9" s="15" t="s">
         <v>16</v>
@@ -1054,30 +1068,32 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B10" s="14" t="s">
         <v>14</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D10" s="13" t="n">
         <v>0.333333333333333</v>
       </c>
-      <c r="E10" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="F10" s="15"/>
-      <c r="G10" s="13"/>
+      <c r="E10" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="F10" s="14"/>
+      <c r="G10" s="13" t="n">
+        <v>0.152777777777778</v>
+      </c>
       <c r="H10" s="14" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="I10" s="14" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="J10" s="13" t="n">
-        <v>0.291666666666667</v>
+        <v>0.260416666666667</v>
       </c>
       <c r="K10" s="15" t="s">
         <v>16</v>
@@ -1092,28 +1108,30 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="13"/>
-      <c r="E11" s="14"/>
+      <c r="E11" s="14" t="s">
+        <v>14</v>
+      </c>
       <c r="F11" s="14" t="s">
         <v>23</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.236111111111111</v>
+        <v>0.284722222222222</v>
       </c>
       <c r="H11" s="14" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="I11" s="14" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J11" s="13" t="n">
-        <v>0.291666666666667</v>
+        <v>0.284722222222222</v>
       </c>
       <c r="K11" s="15" t="s">
         <v>16</v>
@@ -1128,37 +1146,35 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B12" s="17" t="s">
         <v>14</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="D12" s="18" t="n">
-        <v>0.333333333333333</v>
+        <v>0.361111111111111</v>
       </c>
       <c r="E12" s="19" t="s">
         <v>16</v>
       </c>
       <c r="F12" s="19"/>
       <c r="G12" s="18"/>
-      <c r="H12" s="17" t="s">
+      <c r="H12" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="I12" s="19"/>
+      <c r="J12" s="18"/>
+      <c r="K12" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="I12" s="17"/>
-      <c r="J12" s="18" t="n">
-        <v>0.166666666666667</v>
-      </c>
-      <c r="K12" s="17" t="s">
-        <v>32</v>
-      </c>
       <c r="L12" s="17" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="M12" s="18" t="n">
-        <v>0.354166666666667</v>
+        <v>0.319444444444444</v>
       </c>
       <c r="N12" s="19" t="s">
         <v>16</v>
@@ -1168,35 +1184,37 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="B13" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="C13" s="19"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="F13" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="G13" s="18" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="H13" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="I13" s="19"/>
-      <c r="J13" s="18"/>
+      <c r="B13" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" s="18" t="n">
+        <v>0.305555555555556</v>
+      </c>
+      <c r="E13" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="F13" s="19"/>
+      <c r="G13" s="18"/>
+      <c r="H13" s="17"/>
+      <c r="I13" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="J13" s="18" t="n">
+        <v>0.211805555555556</v>
+      </c>
       <c r="K13" s="17" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="L13" s="17" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="M13" s="18" t="n">
-        <v>0.270833333333333</v>
+        <v>0.305555555555556</v>
       </c>
       <c r="N13" s="19" t="s">
         <v>16</v>
@@ -1206,18 +1224,18 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B14" s="20" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C14" s="20"/>
       <c r="D14" s="21" t="n">
         <f aca="false">SUM(D7:D13)</f>
-        <v>1.125</v>
+        <v>1.45833333333333</v>
       </c>
       <c r="E14" s="20" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="F14" s="20"/>
       <c r="G14" s="22" t="n">
@@ -1225,7 +1243,7 @@
         <v>1.45833333333333</v>
       </c>
       <c r="H14" s="20" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="I14" s="20"/>
       <c r="J14" s="23" t="n">
@@ -1233,7 +1251,7 @@
         <v>1.04166666666667</v>
       </c>
       <c r="K14" s="20" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="L14" s="20"/>
       <c r="M14" s="24" t="n">
@@ -1241,7 +1259,7 @@
         <v>0.625</v>
       </c>
       <c r="N14" s="20" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="O14" s="20"/>
       <c r="P14" s="25" t="n">
@@ -1251,7 +1269,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1334,7 +1352,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="B19" s="15" t="s">
         <v>16</v>
@@ -1345,17 +1363,19 @@
         <v>14</v>
       </c>
       <c r="F19" s="14" t="s">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="G19" s="13" t="n">
         <v>0.291666666666667</v>
       </c>
-      <c r="H19" s="14"/>
+      <c r="H19" s="14" t="s">
+        <v>29</v>
+      </c>
       <c r="I19" s="14" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J19" s="13" t="n">
-        <v>0.236111111111111</v>
+        <v>0.260416666666667</v>
       </c>
       <c r="K19" s="15" t="s">
         <v>16</v>
@@ -1370,22 +1390,22 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B20" s="14" t="s">
         <v>14</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="D20" s="13" t="n">
         <v>0.291666666666667</v>
       </c>
       <c r="E20" s="14" t="s">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="F20" s="14" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G20" s="13" t="n">
         <v>0.291666666666667</v>
@@ -1408,7 +1428,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="B21" s="15" t="s">
         <v>16</v>
@@ -1419,17 +1439,19 @@
         <v>14</v>
       </c>
       <c r="F21" s="14" t="s">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="G21" s="13" t="n">
         <v>0.291666666666667</v>
       </c>
-      <c r="H21" s="14"/>
+      <c r="H21" s="14" t="s">
+        <v>29</v>
+      </c>
       <c r="I21" s="14" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J21" s="13" t="n">
-        <v>0.236111111111111</v>
+        <v>0.260416666666667</v>
       </c>
       <c r="K21" s="15" t="s">
         <v>16</v>
@@ -1444,13 +1466,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="B22" s="14" t="s">
         <v>14</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="D22" s="13" t="n">
         <v>0.291666666666667</v>
@@ -1460,12 +1482,14 @@
       </c>
       <c r="F22" s="15"/>
       <c r="G22" s="13"/>
-      <c r="H22" s="14"/>
+      <c r="H22" s="14" t="s">
+        <v>29</v>
+      </c>
       <c r="I22" s="14" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J22" s="13" t="n">
-        <v>0.236111111111111</v>
+        <v>0.260416666666667</v>
       </c>
       <c r="K22" s="15" t="s">
         <v>16</v>
@@ -1480,33 +1504,31 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="B23" s="14" t="s">
         <v>14</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="D23" s="13" t="n">
         <v>0.291666666666667</v>
       </c>
       <c r="E23" s="14" t="s">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="F23" s="14" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G23" s="13" t="n">
         <v>0.291666666666667</v>
       </c>
-      <c r="H23" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="I23" s="14"/>
-      <c r="J23" s="13" t="n">
-        <v>0.0972222222222222</v>
-      </c>
+      <c r="H23" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="I23" s="15"/>
+      <c r="J23" s="13"/>
       <c r="K23" s="15" t="s">
         <v>16</v>
       </c>
@@ -1520,13 +1542,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="16" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="B24" s="17" t="s">
         <v>14</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="D24" s="18" t="n">
         <v>0.291666666666667</v>
@@ -1536,15 +1558,17 @@
       </c>
       <c r="F24" s="19"/>
       <c r="G24" s="18"/>
-      <c r="H24" s="17"/>
+      <c r="H24" s="17" t="s">
+        <v>29</v>
+      </c>
       <c r="I24" s="17" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J24" s="18" t="n">
-        <v>0.236111111111111</v>
+        <v>0.260416666666667</v>
       </c>
       <c r="K24" s="26" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="L24" s="26"/>
       <c r="M24" s="18"/>
@@ -1556,22 +1580,22 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="16" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B25" s="17" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C25" s="17" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D25" s="18" t="n">
         <v>0.291666666666667</v>
       </c>
       <c r="E25" s="17" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="F25" s="17" t="s">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="G25" s="18" t="n">
         <v>0.291666666666667</v>
@@ -1582,7 +1606,7 @@
       <c r="I25" s="19"/>
       <c r="J25" s="18"/>
       <c r="K25" s="26" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="L25" s="26"/>
       <c r="M25" s="18"/>
@@ -1594,10 +1618,10 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C26" s="20"/>
       <c r="D26" s="21" t="n">
@@ -1605,7 +1629,7 @@
         <v>1.45833333333333</v>
       </c>
       <c r="E26" s="20" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="F26" s="20"/>
       <c r="G26" s="22" t="n">
@@ -1613,7 +1637,7 @@
         <v>1.45833333333333</v>
       </c>
       <c r="H26" s="20" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="I26" s="20"/>
       <c r="J26" s="23" t="n">
@@ -1621,7 +1645,7 @@
         <v>1.04166666666667</v>
       </c>
       <c r="K26" s="20" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="L26" s="20"/>
       <c r="M26" s="24" t="n">
@@ -1629,7 +1653,7 @@
         <v>0</v>
       </c>
       <c r="N26" s="20" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="O26" s="20"/>
       <c r="P26" s="25" t="n">
@@ -1639,7 +1663,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1722,7 +1746,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="11" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="B31" s="15" t="s">
         <v>16</v>
@@ -1733,17 +1757,19 @@
         <v>14</v>
       </c>
       <c r="F31" s="14" t="s">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="G31" s="13" t="n">
         <v>0.291666666666667</v>
       </c>
-      <c r="H31" s="14"/>
+      <c r="H31" s="14" t="s">
+        <v>29</v>
+      </c>
       <c r="I31" s="14" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J31" s="13" t="n">
-        <v>0.236111111111111</v>
+        <v>0.260416666666667</v>
       </c>
       <c r="K31" s="15" t="s">
         <v>16</v>
@@ -1758,22 +1784,22 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="11" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B32" s="14" t="s">
         <v>14</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="D32" s="13" t="n">
         <v>0.291666666666667</v>
       </c>
       <c r="E32" s="14" t="s">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="F32" s="14" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G32" s="13" t="n">
         <v>0.291666666666667</v>
@@ -1796,13 +1822,13 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D33" s="13" t="n">
         <v>0.291666666666667</v>
@@ -1811,7 +1837,7 @@
         <v>14</v>
       </c>
       <c r="F33" s="14" t="s">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="G33" s="13" t="n">
         <v>0.291666666666667</v>
@@ -1834,13 +1860,13 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="11" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="B34" s="14" t="s">
         <v>14</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="D34" s="13" t="n">
         <v>0.291666666666667</v>
@@ -1851,13 +1877,13 @@
       <c r="F34" s="15"/>
       <c r="G34" s="13"/>
       <c r="H34" s="14" t="s">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="I34" s="14" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="J34" s="13" t="n">
-        <v>0.284722222222222</v>
+        <v>0.260416666666667</v>
       </c>
       <c r="K34" s="15" t="s">
         <v>16</v>
@@ -1872,34 +1898,34 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B35" s="14" t="s">
         <v>14</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="D35" s="13" t="n">
         <v>0.291666666666667</v>
       </c>
       <c r="E35" s="14" t="s">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="F35" s="14" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G35" s="13" t="n">
         <v>0.291666666666667</v>
       </c>
       <c r="H35" s="14" t="s">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="I35" s="14" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J35" s="13" t="n">
-        <v>0.284722222222222</v>
+        <v>0.260416666666667</v>
       </c>
       <c r="K35" s="15" t="s">
         <v>16</v>
@@ -1914,38 +1940,38 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="16" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B36" s="17" t="s">
         <v>14</v>
       </c>
       <c r="C36" s="17" t="s">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="D36" s="18" t="n">
         <v>0.291666666666667</v>
       </c>
       <c r="E36" s="17" t="s">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="F36" s="17" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G36" s="18" t="n">
         <v>0.291666666666667</v>
       </c>
       <c r="H36" s="26" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="I36" s="26"/>
       <c r="J36" s="18" t="n">
-        <v>0.236111111111111</v>
+        <v>0.260416666666667</v>
       </c>
       <c r="K36" s="17" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="L36" s="17" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="M36" s="18" t="n">
         <v>0.333333333333333</v>
@@ -1958,40 +1984,40 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="16" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B37" s="26" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C37" s="26"/>
       <c r="D37" s="18"/>
       <c r="E37" s="26" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="F37" s="26"/>
       <c r="G37" s="18"/>
       <c r="H37" s="26" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="I37" s="26"/>
       <c r="J37" s="18"/>
       <c r="K37" s="26" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="L37" s="26"/>
       <c r="M37" s="18"/>
       <c r="N37" s="26" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="O37" s="26"/>
       <c r="P37" s="18"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="11" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C38" s="20"/>
       <c r="D38" s="21" t="n">
@@ -1999,7 +2025,7 @@
         <v>1.45833333333333</v>
       </c>
       <c r="E38" s="20" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="F38" s="20"/>
       <c r="G38" s="22" t="n">
@@ -2007,7 +2033,7 @@
         <v>1.45833333333333</v>
       </c>
       <c r="H38" s="20" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="I38" s="20"/>
       <c r="J38" s="23" t="n">
@@ -2015,7 +2041,7 @@
         <v>1.04166666666667</v>
       </c>
       <c r="K38" s="20" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="L38" s="20"/>
       <c r="M38" s="24" t="n">
@@ -2023,7 +2049,7 @@
         <v>0.333333333333333</v>
       </c>
       <c r="N38" s="20" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="O38" s="20"/>
       <c r="P38" s="25" t="n">
@@ -2033,47 +2059,47 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="27" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="28" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="28" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="28" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="28" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="28" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="28" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="28" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="28" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Planning semaine 1 : intérimaire réduit à 10h (12h-17h lun 12 et mar 13)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017sABE5Ku13TMCaT7NQhVkc
</commit_message>
<xml_diff>
--- a/Planning_12oct-1nov.xlsx
+++ b/Planning_12oct-1nov.xlsx
@@ -1043,16 +1043,14 @@
       </c>
       <c r="B11" s="18" t="inlineStr">
         <is>
-          <t>11:00 – 15:00
-16:00 – 19:00
-7h00</t>
+          <t>12:00 – 17:00
+5h00</t>
         </is>
       </c>
       <c r="C11" s="18" t="inlineStr">
         <is>
-          <t>11:00 – 15:00
-16:00 – 19:00
-7h00</t>
+          <t>12:00 – 17:00
+5h00</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
@@ -1082,7 +1080,7 @@
       </c>
       <c r="I11" s="21" t="inlineStr">
         <is>
-          <t>14h00</t>
+          <t>10h00</t>
         </is>
       </c>
     </row>
@@ -1792,7 +1790,7 @@
     <row r="33" ht="28" customHeight="1">
       <c r="A33" s="28" t="inlineStr">
         <is>
-          <t>• Lun 12 et mar 13 : intérimaire de 11h à 19h. Rose ouvre et ferme (clés) et passe la commande du mardi.</t>
+          <t>• Lun 12 et mar 13 : intérimaire de 12h à 17h (5h × 2 = 10h). Rose ouvre et ferme (clés) et passe la commande du mardi.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Planning : intérimaire mardi 13 de 11h à 16h
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017sABE5Ku13TMCaT7NQhVkc
</commit_message>
<xml_diff>
--- a/Planning_12oct-1nov.xlsx
+++ b/Planning_12oct-1nov.xlsx
@@ -1049,7 +1049,7 @@
       </c>
       <c r="C11" s="18" t="inlineStr">
         <is>
-          <t>12:00 – 17:00
+          <t>11:00 – 16:00
 5h00</t>
         </is>
       </c>
@@ -1790,7 +1790,7 @@
     <row r="33" ht="28" customHeight="1">
       <c r="A33" s="28" t="inlineStr">
         <is>
-          <t>• Lun 12 et mar 13 : intérimaire de 12h à 17h (5h × 2 = 10h). Rose ouvre et ferme (clés) et passe la commande du mardi.</t>
+          <t>• Lun 12 et mar 13 : intérimaire lun 12h-17h et mar 11h-16h (5h × 2 = 10h). Rose ouvre et ferme (clés) et passe la commande du mardi.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Planning semaine 3 : 1er novembre planifié normalement, jour férié non travaillé pour les salariés prévus
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017sABE5Ku13TMCaT7NQhVkc
</commit_message>
<xml_diff>
--- a/Planning_12oct-1nov.xlsx
+++ b/Planning_12oct-1nov.xlsx
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1517,97 +1517,95 @@
 7h00</t>
         </is>
       </c>
-      <c r="D24" s="20" t="inlineStr">
+      <c r="D24" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="E24" s="14" t="inlineStr">
+        <is>
+          <t>09:50 – 14:00
+15:00 – 17:50
+7h00</t>
+        </is>
+      </c>
+      <c r="F24" s="14" t="inlineStr">
+        <is>
+          <t>09:50 – 14:00
+15:00 – 17:50
+7h00</t>
+        </is>
+      </c>
+      <c r="G24" s="14" t="inlineStr">
+        <is>
+          <t>09:50 – 14:00
+15:00 – 17:50
+7h00</t>
+        </is>
+      </c>
+      <c r="H24" s="26" t="inlineStr">
+        <is>
+          <t>Férié
+non travaillé
+7h00</t>
+        </is>
+      </c>
+      <c r="I24" s="17" t="inlineStr">
+        <is>
+          <t>35h00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="58" customHeight="1">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>Rose
+contrat 35h</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>09:50 – 14:00
+15:00 – 17:50
+7h00</t>
+        </is>
+      </c>
+      <c r="C25" s="20" t="inlineStr">
         <is>
           <t>11:40 – 15:00
 16:00 – 19:40
 7h00</t>
         </is>
       </c>
-      <c r="E24" s="14" t="inlineStr">
+      <c r="D25" s="14" t="inlineStr">
         <is>
           <t>09:50 – 14:00
 15:00 – 17:50
 7h00</t>
         </is>
       </c>
-      <c r="F24" s="14" t="inlineStr">
-        <is>
-          <t>09:50 – 14:00
-15:00 – 17:50
-7h00</t>
-        </is>
-      </c>
-      <c r="G24" s="14" t="inlineStr">
-        <is>
-          <t>09:50 – 14:00
-15:00 – 17:50
-7h00</t>
-        </is>
-      </c>
-      <c r="H24" s="26" t="inlineStr">
-        <is>
-          <t>FERMÉ
-Toussaint</t>
-        </is>
-      </c>
-      <c r="I24" s="17" t="inlineStr">
-        <is>
-          <t>35h00</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="58" customHeight="1">
-      <c r="A25" s="12" t="inlineStr">
-        <is>
-          <t>Rose
-contrat 35h</t>
-        </is>
-      </c>
-      <c r="B25" s="14" t="inlineStr">
-        <is>
-          <t>09:50 – 14:00
-15:00 – 17:50
-7h00</t>
-        </is>
-      </c>
-      <c r="C25" s="20" t="inlineStr">
+      <c r="E25" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="F25" s="20" t="inlineStr">
         <is>
           <t>11:40 – 15:00
 16:00 – 19:40
 7h00</t>
         </is>
       </c>
-      <c r="D25" s="14" t="inlineStr">
-        <is>
-          <t>09:50 – 14:00
-15:00 – 17:50
-7h00</t>
-        </is>
-      </c>
-      <c r="E25" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="F25" s="20" t="inlineStr">
-        <is>
-          <t>11:40 – 15:00
-16:00 – 19:40
-7h00</t>
-        </is>
-      </c>
-      <c r="G25" s="20" t="inlineStr">
-        <is>
-          <t>11:40 – 15:00
-16:00 – 19:40
-7h00</t>
+      <c r="G25" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
         </is>
       </c>
       <c r="H25" s="26" t="inlineStr">
         <is>
-          <t>FERMÉ
-Toussaint</t>
+          <t>Férié
+non travaillé
+7h00</t>
         </is>
       </c>
       <c r="I25" s="17" t="inlineStr">
@@ -1635,35 +1633,35 @@
           <t>Repos</t>
         </is>
       </c>
-      <c r="D26" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="E26" s="20" t="inlineStr">
+      <c r="D26" s="20" t="inlineStr">
         <is>
           <t>12:25 – 15:00
 16:00 – 19:40
 6h15</t>
         </is>
       </c>
-      <c r="F26" s="20" t="inlineStr">
+      <c r="E26" s="20" t="inlineStr">
         <is>
           <t>12:25 – 15:00
 16:00 – 19:40
 6h15</t>
         </is>
       </c>
+      <c r="F26" s="20" t="inlineStr">
+        <is>
+          <t>12:25 – 15:00
+16:00 – 19:40
+6h15</t>
+        </is>
+      </c>
       <c r="G26" s="15" t="inlineStr">
         <is>
-          <t>Congé
-6h15</t>
-        </is>
-      </c>
-      <c r="H26" s="26" t="inlineStr">
-        <is>
-          <t>FERMÉ
-Toussaint</t>
+          <t>Congé</t>
+        </is>
+      </c>
+      <c r="H26" s="15" t="inlineStr">
+        <is>
+          <t>Congé</t>
         </is>
       </c>
       <c r="I26" s="17" t="inlineStr">
@@ -1706,20 +1704,21 @@
       </c>
       <c r="G27" s="20" t="inlineStr">
         <is>
-          <t>10:40 – 15:00
+          <t>11:00 – 15:00
 16:00 – 19:40
-8h00</t>
+7h40</t>
         </is>
       </c>
       <c r="H27" s="26" t="inlineStr">
         <is>
-          <t>FERMÉ
-Toussaint</t>
-        </is>
-      </c>
-      <c r="I27" s="25" t="inlineStr">
-        <is>
-          <t>8h00</t>
+          <t>Férié
+non travaillé
+7h20</t>
+        </is>
+      </c>
+      <c r="I27" s="17" t="inlineStr">
+        <is>
+          <t>15h00</t>
         </is>
       </c>
     </row>
@@ -1756,12 +1755,12 @@
       </c>
       <c r="G28" s="23" t="inlineStr">
         <is>
-          <t>3 pers.</t>
+          <t>2 pers.</t>
         </is>
       </c>
       <c r="H28" s="23" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Fermé (férié)</t>
         </is>
       </c>
       <c r="I28" s="24" t="n"/>
@@ -1776,7 +1775,7 @@
     <row r="31" ht="28" customHeight="1">
       <c r="A31" s="28" t="inlineStr">
         <is>
-          <t>• Dimanche : Yassine + Sara + Rose ou Jennyfer en alternance (18/10 Jennyfer, 25/10 Rose). Jennyfer est toujours en fermeture.</t>
+          <t>• Dimanche : Yassine + Sara + Rose ou Jennyfer en alternance (18/10 Jennyfer, 25/10 Rose, 1/11 Rose car Jennyfer en congé). Jennyfer est toujours en fermeture.</t>
         </is>
       </c>
     </row>
@@ -1804,15 +1803,23 @@
     <row r="35" ht="28" customHeight="1">
       <c r="A35" s="28" t="inlineStr">
         <is>
-          <t>• Sara indispo sam 24 + dim 25 · Jennyfer en congé du 31/10 au 2/11 (6h15 décomptées) · Dimanche 1er novembre (Toussaint) : magasin fermé.</t>
+          <t>• Sara indispo sam 24 + dim 25 · Jennyfer en congé du 31/10 au 2/11 (ses jours de travail de la semaine ne tombent pas dessus : 25h).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="28" customHeight="1">
+      <c r="A36" s="28" t="inlineStr">
+        <is>
+          <t>• Dim 1er novembre (Toussaint) : planning normal (Yassine + Sara + Rose), mais le jour férié tombe sur leur journée → ils ne travaillent pas, les heures prévues sont comptées (férié chômé). Pour Sara (moins de 3 mois d'ancienneté), le paiement de ce jour n'est pas garanti par la loi : à vérifier avec la paie.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A33:I33"/>
     <mergeCell ref="A5:I5"/>
     <mergeCell ref="A32:I32"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A14:I14"/>
     <mergeCell ref="A31:I31"/>
     <mergeCell ref="A22:I22"/>

</xml_diff>

<commit_message>
Planning 19/10-1/11 refait : Rose en ouverture, Jennyfer en fermeture, Yassine fermeture/milieu, dimanches à 2
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017sABE5Ku13TMCaT7NQhVkc
</commit_message>
<xml_diff>
--- a/Planning_12oct-1nov.xlsx
+++ b/Planning_12oct-1nov.xlsx
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1188,9 +1188,11 @@
 contrat 35h</t>
         </is>
       </c>
-      <c r="B16" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
+      <c r="B16" s="20" t="inlineStr">
+        <is>
+          <t>11:40 – 15:00
+16:00 – 19:40
+7h00</t>
         </is>
       </c>
       <c r="C16" s="14" t="inlineStr">
@@ -1205,90 +1207,88 @@
           <t>Repos</t>
         </is>
       </c>
-      <c r="E16" s="14" t="inlineStr">
+      <c r="E16" s="20" t="inlineStr">
+        <is>
+          <t>11:40 – 15:00
+16:00 – 19:40
+7h00</t>
+        </is>
+      </c>
+      <c r="F16" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="G16" s="20" t="inlineStr">
+        <is>
+          <t>11:40 – 15:00
+16:00 – 19:40
+7h00</t>
+        </is>
+      </c>
+      <c r="H16" s="14" t="inlineStr">
+        <is>
+          <t>10:50 – 14:00
+15:00 – 18:50
+7h00</t>
+        </is>
+      </c>
+      <c r="I16" s="17" t="inlineStr">
+        <is>
+          <t>35h00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="58" customHeight="1">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>Rose
+contrat 35h</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
         <is>
           <t>09:50 – 14:00
 15:00 – 17:50
 7h00</t>
         </is>
       </c>
-      <c r="F16" s="14" t="inlineStr">
+      <c r="C17" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
         <is>
           <t>09:50 – 14:00
 15:00 – 17:50
 7h00</t>
         </is>
       </c>
-      <c r="G16" s="14" t="inlineStr">
+      <c r="E17" s="14" t="inlineStr">
         <is>
           <t>09:50 – 14:00
 15:00 – 17:50
 7h00</t>
         </is>
       </c>
-      <c r="H16" s="14" t="inlineStr">
-        <is>
-          <t>10:50 – 14:00
-15:00 – 18:50
-7h00</t>
-        </is>
-      </c>
-      <c r="I16" s="17" t="inlineStr">
-        <is>
-          <t>35h00</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="58" customHeight="1">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t>Rose
-contrat 35h</t>
-        </is>
-      </c>
-      <c r="B17" s="14" t="inlineStr">
+      <c r="F17" s="14" t="inlineStr">
         <is>
           <t>09:50 – 14:00
 15:00 – 17:50
 7h00</t>
         </is>
       </c>
-      <c r="C17" s="20" t="inlineStr">
-        <is>
-          <t>11:40 – 15:00
-16:00 – 19:40
-7h00</t>
-        </is>
-      </c>
-      <c r="D17" s="14" t="inlineStr">
+      <c r="G17" s="14" t="inlineStr">
         <is>
           <t>09:50 – 14:00
 15:00 – 17:50
 7h00</t>
         </is>
       </c>
-      <c r="E17" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="F17" s="20" t="inlineStr">
-        <is>
-          <t>11:40 – 15:00
-16:00 – 19:40
-7h00</t>
-        </is>
-      </c>
-      <c r="G17" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="H17" s="20" t="inlineStr">
-        <is>
-          <t>11:10 – 15:00
-16:00 – 19:10
-7h00</t>
+      <c r="H17" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
         </is>
       </c>
       <c r="I17" s="17" t="inlineStr">
@@ -1304,18 +1304,18 @@
 contrat 25h</t>
         </is>
       </c>
-      <c r="B18" s="20" t="inlineStr">
+      <c r="B18" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="C18" s="20" t="inlineStr">
         <is>
           <t>12:25 – 15:00
 16:00 – 19:40
 6h15</t>
         </is>
       </c>
-      <c r="C18" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
       <c r="D18" s="20" t="inlineStr">
         <is>
           <t>12:25 – 15:00
@@ -1323,337 +1323,337 @@
 6h15</t>
         </is>
       </c>
-      <c r="E18" s="20" t="inlineStr">
+      <c r="E18" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="F18" s="20" t="inlineStr">
         <is>
           <t>12:25 – 15:00
 16:00 – 19:40
 6h15</t>
         </is>
       </c>
-      <c r="F18" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="G18" s="20" t="inlineStr">
+      <c r="G18" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="H18" s="20" t="inlineStr">
+        <is>
+          <t>11:55 – 15:00
+16:00 – 19:10
+6h15</t>
+        </is>
+      </c>
+      <c r="I18" s="17" t="inlineStr">
+        <is>
+          <t>25h00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="58" customHeight="1">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>Sara
+contrat 15h</t>
+        </is>
+      </c>
+      <c r="B19" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="C19" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="E19" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="F19" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="G19" s="15" t="inlineStr">
+        <is>
+          <t>Indispo</t>
+        </is>
+      </c>
+      <c r="H19" s="15" t="inlineStr">
+        <is>
+          <t>Indispo</t>
+        </is>
+      </c>
+      <c r="I19" s="25" t="inlineStr">
+        <is>
+          <t>0h00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="22" t="inlineStr">
+        <is>
+          <t>Présents</t>
+        </is>
+      </c>
+      <c r="B20" s="23" t="inlineStr">
+        <is>
+          <t>2 pers.</t>
+        </is>
+      </c>
+      <c r="C20" s="23" t="inlineStr">
+        <is>
+          <t>2 pers.</t>
+        </is>
+      </c>
+      <c r="D20" s="23" t="inlineStr">
+        <is>
+          <t>2 pers.</t>
+        </is>
+      </c>
+      <c r="E20" s="23" t="inlineStr">
+        <is>
+          <t>2 pers.</t>
+        </is>
+      </c>
+      <c r="F20" s="23" t="inlineStr">
+        <is>
+          <t>2 pers.</t>
+        </is>
+      </c>
+      <c r="G20" s="23" t="inlineStr">
+        <is>
+          <t>2 pers.</t>
+        </is>
+      </c>
+      <c r="H20" s="23" t="inlineStr">
+        <is>
+          <t>2 pers.</t>
+        </is>
+      </c>
+      <c r="I20" s="24" t="n"/>
+    </row>
+    <row r="22" ht="26" customHeight="1">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>SEMAINE 3  ·  du lundi 26 octobre au dimanche 1 novembre</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>Salarié</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Lun 26/10</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>Mar 27/10</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>Mer 28/10</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>Jeu 29/10</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>Ven 30/10</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="inlineStr">
+        <is>
+          <t>Sam 31/10</t>
+        </is>
+      </c>
+      <c r="H23" s="11" t="inlineStr">
+        <is>
+          <t>Dim 01/11</t>
+        </is>
+      </c>
+      <c r="I23" s="11" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="58" customHeight="1">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>Yassine
+contrat 35h</t>
+        </is>
+      </c>
+      <c r="B24" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="inlineStr">
+        <is>
+          <t>09:50 – 14:00
+15:00 – 17:50
+7h00</t>
+        </is>
+      </c>
+      <c r="D24" s="20" t="inlineStr">
+        <is>
+          <t>11:40 – 15:00
+16:00 – 19:40
+7h00</t>
+        </is>
+      </c>
+      <c r="E24" s="18" t="inlineStr">
+        <is>
+          <t>11:00 – 14:00
+15:00 – 19:00
+7h00</t>
+        </is>
+      </c>
+      <c r="F24" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="G24" s="20" t="inlineStr">
+        <is>
+          <t>11:40 – 15:00
+16:00 – 19:40
+7h00</t>
+        </is>
+      </c>
+      <c r="H24" s="26" t="inlineStr">
+        <is>
+          <t>Férié
+non travaillé
+7h00</t>
+        </is>
+      </c>
+      <c r="I24" s="17" t="inlineStr">
+        <is>
+          <t>35h00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="58" customHeight="1">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>Rose
+contrat 35h</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>09:50 – 14:00
+15:00 – 17:50
+7h00</t>
+        </is>
+      </c>
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>09:50 – 14:00
+15:00 – 17:50
+7h00</t>
+        </is>
+      </c>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>09:50 – 14:00
+15:00 – 17:50
+7h00</t>
+        </is>
+      </c>
+      <c r="E25" s="14" t="inlineStr">
+        <is>
+          <t>09:50 – 14:00
+15:00 – 17:50
+7h00</t>
+        </is>
+      </c>
+      <c r="F25" s="14" t="inlineStr">
+        <is>
+          <t>09:50 – 14:00
+15:00 – 17:50
+7h00</t>
+        </is>
+      </c>
+      <c r="G25" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="H25" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="I25" s="17" t="inlineStr">
+        <is>
+          <t>35h00</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="58" customHeight="1">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>Jennyfer
+contrat 25h</t>
+        </is>
+      </c>
+      <c r="B26" s="20" t="inlineStr">
         <is>
           <t>12:25 – 15:00
 16:00 – 19:40
 6h15</t>
         </is>
       </c>
-      <c r="H18" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="I18" s="17" t="inlineStr">
-        <is>
-          <t>25h00</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="58" customHeight="1">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>Sara
-contrat 15h</t>
-        </is>
-      </c>
-      <c r="B19" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="C19" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="D19" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="E19" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="F19" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="G19" s="15" t="inlineStr">
-        <is>
-          <t>Indispo</t>
-        </is>
-      </c>
-      <c r="H19" s="15" t="inlineStr">
-        <is>
-          <t>Indispo</t>
-        </is>
-      </c>
-      <c r="I19" s="25" t="inlineStr">
-        <is>
-          <t>0h00</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="22" t="inlineStr">
-        <is>
-          <t>Présents</t>
-        </is>
-      </c>
-      <c r="B20" s="23" t="inlineStr">
-        <is>
-          <t>2 pers.</t>
-        </is>
-      </c>
-      <c r="C20" s="23" t="inlineStr">
-        <is>
-          <t>2 pers.</t>
-        </is>
-      </c>
-      <c r="D20" s="23" t="inlineStr">
-        <is>
-          <t>2 pers.</t>
-        </is>
-      </c>
-      <c r="E20" s="23" t="inlineStr">
-        <is>
-          <t>2 pers.</t>
-        </is>
-      </c>
-      <c r="F20" s="23" t="inlineStr">
-        <is>
-          <t>2 pers.</t>
-        </is>
-      </c>
-      <c r="G20" s="23" t="inlineStr">
-        <is>
-          <t>2 pers.</t>
-        </is>
-      </c>
-      <c r="H20" s="23" t="inlineStr">
-        <is>
-          <t>2 pers.</t>
-        </is>
-      </c>
-      <c r="I20" s="24" t="n"/>
-    </row>
-    <row r="22" ht="26" customHeight="1">
-      <c r="A22" s="10" t="inlineStr">
-        <is>
-          <t>SEMAINE 3  ·  du lundi 26 octobre au dimanche 1 novembre</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="11" t="inlineStr">
-        <is>
-          <t>Salarié</t>
-        </is>
-      </c>
-      <c r="B23" s="11" t="inlineStr">
-        <is>
-          <t>Lun 26/10</t>
-        </is>
-      </c>
-      <c r="C23" s="11" t="inlineStr">
-        <is>
-          <t>Mar 27/10</t>
-        </is>
-      </c>
-      <c r="D23" s="11" t="inlineStr">
-        <is>
-          <t>Mer 28/10</t>
-        </is>
-      </c>
-      <c r="E23" s="11" t="inlineStr">
-        <is>
-          <t>Jeu 29/10</t>
-        </is>
-      </c>
-      <c r="F23" s="11" t="inlineStr">
-        <is>
-          <t>Ven 30/10</t>
-        </is>
-      </c>
-      <c r="G23" s="11" t="inlineStr">
-        <is>
-          <t>Sam 31/10</t>
-        </is>
-      </c>
-      <c r="H23" s="11" t="inlineStr">
-        <is>
-          <t>Dim 01/11</t>
-        </is>
-      </c>
-      <c r="I23" s="11" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="58" customHeight="1">
-      <c r="A24" s="12" t="inlineStr">
-        <is>
-          <t>Yassine
-contrat 35h</t>
-        </is>
-      </c>
-      <c r="B24" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="C24" s="14" t="inlineStr">
-        <is>
-          <t>09:50 – 14:00
-15:00 – 17:50
-7h00</t>
-        </is>
-      </c>
-      <c r="D24" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="E24" s="14" t="inlineStr">
-        <is>
-          <t>09:50 – 14:00
-15:00 – 17:50
-7h00</t>
-        </is>
-      </c>
-      <c r="F24" s="14" t="inlineStr">
-        <is>
-          <t>09:50 – 14:00
-15:00 – 17:50
-7h00</t>
-        </is>
-      </c>
-      <c r="G24" s="14" t="inlineStr">
-        <is>
-          <t>09:50 – 14:00
-15:00 – 17:50
-7h00</t>
-        </is>
-      </c>
-      <c r="H24" s="26" t="inlineStr">
-        <is>
-          <t>Férié
-non travaillé
-7h00</t>
-        </is>
-      </c>
-      <c r="I24" s="17" t="inlineStr">
-        <is>
-          <t>35h00</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="58" customHeight="1">
-      <c r="A25" s="12" t="inlineStr">
-        <is>
-          <t>Rose
-contrat 35h</t>
-        </is>
-      </c>
-      <c r="B25" s="14" t="inlineStr">
-        <is>
-          <t>09:50 – 14:00
-15:00 – 17:50
-7h00</t>
-        </is>
-      </c>
-      <c r="C25" s="20" t="inlineStr">
-        <is>
-          <t>11:40 – 15:00
-16:00 – 19:40
-7h00</t>
-        </is>
-      </c>
-      <c r="D25" s="14" t="inlineStr">
-        <is>
-          <t>09:50 – 14:00
-15:00 – 17:50
-7h00</t>
-        </is>
-      </c>
-      <c r="E25" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="F25" s="20" t="inlineStr">
-        <is>
-          <t>11:40 – 15:00
-16:00 – 19:40
-7h00</t>
-        </is>
-      </c>
-      <c r="G25" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="H25" s="26" t="inlineStr">
-        <is>
-          <t>Férié
-non travaillé
-7h00</t>
-        </is>
-      </c>
-      <c r="I25" s="17" t="inlineStr">
-        <is>
-          <t>35h00</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="58" customHeight="1">
-      <c r="A26" s="12" t="inlineStr">
-        <is>
-          <t>Jennyfer
-contrat 25h</t>
-        </is>
-      </c>
-      <c r="B26" s="20" t="inlineStr">
+      <c r="C26" s="20" t="inlineStr">
         <is>
           <t>12:25 – 15:00
 16:00 – 19:40
 6h15</t>
         </is>
       </c>
-      <c r="C26" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="D26" s="20" t="inlineStr">
+      <c r="D26" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="E26" s="20" t="inlineStr">
         <is>
           <t>12:25 – 15:00
 16:00 – 19:40
 6h15</t>
         </is>
       </c>
-      <c r="E26" s="20" t="inlineStr">
+      <c r="F26" s="20" t="inlineStr">
         <is>
           <t>12:25 – 15:00
 16:00 – 19:40
 6h15</t>
         </is>
       </c>
-      <c r="F26" s="20" t="inlineStr">
-        <is>
-          <t>12:25 – 15:00
-16:00 – 19:40
-6h15</t>
-        </is>
-      </c>
       <c r="G26" s="15" t="inlineStr">
         <is>
           <t>Congé</t>
@@ -1702,10 +1702,10 @@
           <t>Repos</t>
         </is>
       </c>
-      <c r="G27" s="20" t="inlineStr">
-        <is>
-          <t>11:00 – 15:00
-16:00 – 19:40
+      <c r="G27" s="14" t="inlineStr">
+        <is>
+          <t>09:50 – 14:00
+15:00 – 18:30
 7h40</t>
         </is>
       </c>
@@ -1735,22 +1735,22 @@
       </c>
       <c r="C28" s="23" t="inlineStr">
         <is>
+          <t>3 pers.</t>
+        </is>
+      </c>
+      <c r="D28" s="23" t="inlineStr">
+        <is>
           <t>2 pers.</t>
         </is>
       </c>
-      <c r="D28" s="23" t="inlineStr">
+      <c r="E28" s="23" t="inlineStr">
+        <is>
+          <t>3 pers.</t>
+        </is>
+      </c>
+      <c r="F28" s="23" t="inlineStr">
         <is>
           <t>2 pers.</t>
-        </is>
-      </c>
-      <c r="E28" s="23" t="inlineStr">
-        <is>
-          <t>2 pers.</t>
-        </is>
-      </c>
-      <c r="F28" s="23" t="inlineStr">
-        <is>
-          <t>3 pers.</t>
         </is>
       </c>
       <c r="G28" s="23" t="inlineStr">
@@ -1775,51 +1775,43 @@
     <row r="31" ht="28" customHeight="1">
       <c r="A31" s="28" t="inlineStr">
         <is>
-          <t>• Dimanche : Yassine + Sara + Rose ou Jennyfer en alternance (18/10 Jennyfer, 25/10 Rose, 1/11 Rose car Jennyfer en congé). Jennyfer est toujours en fermeture.</t>
+          <t>• Dès le 19/10 : Rose toujours en ouverture, Jennyfer toujours en fermeture, Yassine en fermeture ou milieu de journée ; le mardi Yassine est là dès 09:50 pour la commande (avant 11h).</t>
         </is>
       </c>
     </row>
     <row r="32" ht="28" customHeight="1">
       <c r="A32" s="28" t="inlineStr">
         <is>
-          <t>• Semaine du séminaire : Yassine = 35h (séminaire lun 3h30 + mar 7h30, puis magasin jeu 8h, sam 8h40, dim 7h20). Trajet à récupérer avant fin novembre. Indispo ven 16.</t>
+          <t>• Dimanche à 2 : Sara + Yassine ou Jennyfer en alternance. Le 25/10 Sara est indispo → Yassine + Jennyfer. Le 1/11 → Sara + Yassine (Jennyfer en congé), jour férié non travaillé.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="28" customHeight="1">
       <c r="A33" s="28" t="inlineStr">
         <is>
-          <t>• Lun 12 et mar 13 : intérimaire lun 12h-17h et mar 11h-16h (5h × 2 = 10h). Rose ouvre et ferme (clés) et passe la commande du mardi.</t>
+          <t>• Semaine du séminaire : Yassine = 35h (séminaire lun 3h30 + mar 7h30, puis magasin jeu 8h, sam 8h40, dim 7h20). Indispo ven 16. Intérimaire lun 12h-17h et mar 11h-16h (10h).</t>
         </is>
       </c>
     </row>
     <row r="34" ht="28" customHeight="1">
       <c r="A34" s="28" t="inlineStr">
         <is>
-          <t>• Livraisons : 3 personnes le jeu 15 et le ven 30 ; 2 seulement les ven 16, jeu 22, ven 23, jeu 29 → renfort possible (intérim / heures complémentaires).</t>
+          <t>• Livraisons : 3 personnes le jeu 15 et le jeu 29 ; 2 personnes les ven 16, jeu 22, ven 23, ven 30.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="28" customHeight="1">
       <c r="A35" s="28" t="inlineStr">
         <is>
-          <t>• Sara indispo sam 24 + dim 25 · Jennyfer en congé du 31/10 au 2/11 (ses jours de travail de la semaine ne tombent pas dessus : 25h).</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="28" customHeight="1">
-      <c r="A36" s="28" t="inlineStr">
-        <is>
-          <t>• Dim 1er novembre (Toussaint) : planning normal (Yassine + Sara + Rose), mais le jour férié tombe sur leur journée → ils ne travaillent pas, les heures prévues sont comptées (férié chômé). Pour Sara (moins de 3 mois d'ancienneté), le paiement de ce jour n'est pas garanti par la loi : à vérifier avec la paie.</t>
+          <t>• Sara indispo sam 24 + dim 25 · Jennyfer en congé du 31/10 au 2/11 · Dim 1/11 (Toussaint) : heures prévues comptées (férié chômé) ; pour Sara (&lt; 3 mois d'ancienneté), paiement à vérifier avec la paie.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="8">
     <mergeCell ref="A33:I33"/>
     <mergeCell ref="A5:I5"/>
     <mergeCell ref="A32:I32"/>
-    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A14:I14"/>
     <mergeCell ref="A31:I31"/>
     <mergeCell ref="A22:I22"/>

</xml_diff>

<commit_message>
Semaine du 19/10 : +5h pour Yassine, Rose et Jennyfer (3 personnes les jours de livraison)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017sABE5Ku13TMCaT7NQhVkc
</commit_message>
<xml_diff>
--- a/Planning_12oct-1nov.xlsx
+++ b/Planning_12oct-1nov.xlsx
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1214,9 +1214,10 @@
 7h00</t>
         </is>
       </c>
-      <c r="F16" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>11:00 – 16:00
+5h00</t>
         </is>
       </c>
       <c r="G16" s="20" t="inlineStr">
@@ -1233,9 +1234,9 @@
 7h00</t>
         </is>
       </c>
-      <c r="I16" s="17" t="inlineStr">
-        <is>
-          <t>35h00</t>
+      <c r="I16" s="25" t="inlineStr">
+        <is>
+          <t>40h00</t>
         </is>
       </c>
     </row>
@@ -1247,413 +1248,414 @@
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>09:50 – 14:00
+15:00 – 18:50
+8h00</t>
+        </is>
+      </c>
+      <c r="C17" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>09:50 – 14:00
+15:00 – 18:50
+8h00</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="inlineStr">
+        <is>
+          <t>09:50 – 14:00
+15:00 – 18:50
+8h00</t>
+        </is>
+      </c>
+      <c r="F17" s="14" t="inlineStr">
+        <is>
+          <t>09:50 – 14:00
+15:00 – 18:50
+8h00</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="inlineStr">
+        <is>
+          <t>09:50 – 14:00
+15:00 – 18:50
+8h00</t>
+        </is>
+      </c>
+      <c r="H17" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="I17" s="25" t="inlineStr">
+        <is>
+          <t>40h00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="58" customHeight="1">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Jennyfer
+contrat 25h</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="C18" s="20" t="inlineStr">
+        <is>
+          <t>12:25 – 15:00
+16:00 – 19:40
+6h15</t>
+        </is>
+      </c>
+      <c r="D18" s="20" t="inlineStr">
+        <is>
+          <t>12:25 – 15:00
+16:00 – 19:40
+6h15</t>
+        </is>
+      </c>
+      <c r="E18" s="20" t="inlineStr">
+        <is>
+          <t>14:40 – 19:40
+5h00</t>
+        </is>
+      </c>
+      <c r="F18" s="20" t="inlineStr">
+        <is>
+          <t>12:25 – 15:00
+16:00 – 19:40
+6h15</t>
+        </is>
+      </c>
+      <c r="G18" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="H18" s="20" t="inlineStr">
+        <is>
+          <t>11:55 – 15:00
+16:00 – 19:10
+6h15</t>
+        </is>
+      </c>
+      <c r="I18" s="25" t="inlineStr">
+        <is>
+          <t>30h00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="58" customHeight="1">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>Sara
+contrat 15h</t>
+        </is>
+      </c>
+      <c r="B19" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="C19" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="E19" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="F19" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="G19" s="15" t="inlineStr">
+        <is>
+          <t>Indispo</t>
+        </is>
+      </c>
+      <c r="H19" s="15" t="inlineStr">
+        <is>
+          <t>Indispo</t>
+        </is>
+      </c>
+      <c r="I19" s="25" t="inlineStr">
+        <is>
+          <t>0h00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="22" t="inlineStr">
+        <is>
+          <t>Présents</t>
+        </is>
+      </c>
+      <c r="B20" s="23" t="inlineStr">
+        <is>
+          <t>2 pers.</t>
+        </is>
+      </c>
+      <c r="C20" s="23" t="inlineStr">
+        <is>
+          <t>2 pers.</t>
+        </is>
+      </c>
+      <c r="D20" s="23" t="inlineStr">
+        <is>
+          <t>2 pers.</t>
+        </is>
+      </c>
+      <c r="E20" s="23" t="inlineStr">
+        <is>
+          <t>3 pers.</t>
+        </is>
+      </c>
+      <c r="F20" s="23" t="inlineStr">
+        <is>
+          <t>3 pers.</t>
+        </is>
+      </c>
+      <c r="G20" s="23" t="inlineStr">
+        <is>
+          <t>2 pers.</t>
+        </is>
+      </c>
+      <c r="H20" s="23" t="inlineStr">
+        <is>
+          <t>2 pers.</t>
+        </is>
+      </c>
+      <c r="I20" s="24" t="n"/>
+    </row>
+    <row r="22" ht="26" customHeight="1">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>SEMAINE 3  ·  du lundi 26 octobre au dimanche 1 novembre</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>Salarié</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Lun 26/10</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>Mar 27/10</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>Mer 28/10</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>Jeu 29/10</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>Ven 30/10</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="inlineStr">
+        <is>
+          <t>Sam 31/10</t>
+        </is>
+      </c>
+      <c r="H23" s="11" t="inlineStr">
+        <is>
+          <t>Dim 01/11</t>
+        </is>
+      </c>
+      <c r="I23" s="11" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="58" customHeight="1">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>Yassine
+contrat 35h</t>
+        </is>
+      </c>
+      <c r="B24" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="inlineStr">
         <is>
           <t>09:50 – 14:00
 15:00 – 17:50
 7h00</t>
         </is>
       </c>
-      <c r="C17" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="D17" s="14" t="inlineStr">
+      <c r="D24" s="20" t="inlineStr">
+        <is>
+          <t>11:40 – 15:00
+16:00 – 19:40
+7h00</t>
+        </is>
+      </c>
+      <c r="E24" s="18" t="inlineStr">
+        <is>
+          <t>11:00 – 14:00
+15:00 – 19:00
+7h00</t>
+        </is>
+      </c>
+      <c r="F24" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="G24" s="20" t="inlineStr">
+        <is>
+          <t>11:40 – 15:00
+16:00 – 19:40
+7h00</t>
+        </is>
+      </c>
+      <c r="H24" s="26" t="inlineStr">
+        <is>
+          <t>Férié
+non travaillé
+7h00</t>
+        </is>
+      </c>
+      <c r="I24" s="17" t="inlineStr">
+        <is>
+          <t>35h00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="58" customHeight="1">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>Rose
+contrat 35h</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
         <is>
           <t>09:50 – 14:00
 15:00 – 17:50
 7h00</t>
         </is>
       </c>
-      <c r="E17" s="14" t="inlineStr">
+      <c r="C25" s="14" t="inlineStr">
         <is>
           <t>09:50 – 14:00
 15:00 – 17:50
 7h00</t>
         </is>
       </c>
-      <c r="F17" s="14" t="inlineStr">
+      <c r="D25" s="14" t="inlineStr">
         <is>
           <t>09:50 – 14:00
 15:00 – 17:50
 7h00</t>
         </is>
       </c>
-      <c r="G17" s="14" t="inlineStr">
+      <c r="E25" s="14" t="inlineStr">
         <is>
           <t>09:50 – 14:00
 15:00 – 17:50
 7h00</t>
         </is>
       </c>
-      <c r="H17" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="I17" s="17" t="inlineStr">
+      <c r="F25" s="14" t="inlineStr">
+        <is>
+          <t>09:50 – 14:00
+15:00 – 17:50
+7h00</t>
+        </is>
+      </c>
+      <c r="G25" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="H25" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="I25" s="17" t="inlineStr">
         <is>
           <t>35h00</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="58" customHeight="1">
-      <c r="A18" s="12" t="inlineStr">
+    <row r="26" ht="58" customHeight="1">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t>Jennyfer
 contrat 25h</t>
         </is>
       </c>
-      <c r="B18" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="C18" s="20" t="inlineStr">
+      <c r="B26" s="20" t="inlineStr">
         <is>
           <t>12:25 – 15:00
 16:00 – 19:40
 6h15</t>
         </is>
       </c>
-      <c r="D18" s="20" t="inlineStr">
+      <c r="C26" s="20" t="inlineStr">
         <is>
           <t>12:25 – 15:00
 16:00 – 19:40
 6h15</t>
         </is>
       </c>
-      <c r="E18" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="F18" s="20" t="inlineStr">
+      <c r="D26" s="19" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="E26" s="20" t="inlineStr">
         <is>
           <t>12:25 – 15:00
 16:00 – 19:40
 6h15</t>
         </is>
       </c>
-      <c r="G18" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="H18" s="20" t="inlineStr">
-        <is>
-          <t>11:55 – 15:00
-16:00 – 19:10
-6h15</t>
-        </is>
-      </c>
-      <c r="I18" s="17" t="inlineStr">
-        <is>
-          <t>25h00</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="58" customHeight="1">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>Sara
-contrat 15h</t>
-        </is>
-      </c>
-      <c r="B19" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="C19" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="D19" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="E19" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="F19" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="G19" s="15" t="inlineStr">
-        <is>
-          <t>Indispo</t>
-        </is>
-      </c>
-      <c r="H19" s="15" t="inlineStr">
-        <is>
-          <t>Indispo</t>
-        </is>
-      </c>
-      <c r="I19" s="25" t="inlineStr">
-        <is>
-          <t>0h00</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="22" t="inlineStr">
-        <is>
-          <t>Présents</t>
-        </is>
-      </c>
-      <c r="B20" s="23" t="inlineStr">
-        <is>
-          <t>2 pers.</t>
-        </is>
-      </c>
-      <c r="C20" s="23" t="inlineStr">
-        <is>
-          <t>2 pers.</t>
-        </is>
-      </c>
-      <c r="D20" s="23" t="inlineStr">
-        <is>
-          <t>2 pers.</t>
-        </is>
-      </c>
-      <c r="E20" s="23" t="inlineStr">
-        <is>
-          <t>2 pers.</t>
-        </is>
-      </c>
-      <c r="F20" s="23" t="inlineStr">
-        <is>
-          <t>2 pers.</t>
-        </is>
-      </c>
-      <c r="G20" s="23" t="inlineStr">
-        <is>
-          <t>2 pers.</t>
-        </is>
-      </c>
-      <c r="H20" s="23" t="inlineStr">
-        <is>
-          <t>2 pers.</t>
-        </is>
-      </c>
-      <c r="I20" s="24" t="n"/>
-    </row>
-    <row r="22" ht="26" customHeight="1">
-      <c r="A22" s="10" t="inlineStr">
-        <is>
-          <t>SEMAINE 3  ·  du lundi 26 octobre au dimanche 1 novembre</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="11" t="inlineStr">
-        <is>
-          <t>Salarié</t>
-        </is>
-      </c>
-      <c r="B23" s="11" t="inlineStr">
-        <is>
-          <t>Lun 26/10</t>
-        </is>
-      </c>
-      <c r="C23" s="11" t="inlineStr">
-        <is>
-          <t>Mar 27/10</t>
-        </is>
-      </c>
-      <c r="D23" s="11" t="inlineStr">
-        <is>
-          <t>Mer 28/10</t>
-        </is>
-      </c>
-      <c r="E23" s="11" t="inlineStr">
-        <is>
-          <t>Jeu 29/10</t>
-        </is>
-      </c>
-      <c r="F23" s="11" t="inlineStr">
-        <is>
-          <t>Ven 30/10</t>
-        </is>
-      </c>
-      <c r="G23" s="11" t="inlineStr">
-        <is>
-          <t>Sam 31/10</t>
-        </is>
-      </c>
-      <c r="H23" s="11" t="inlineStr">
-        <is>
-          <t>Dim 01/11</t>
-        </is>
-      </c>
-      <c r="I23" s="11" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="58" customHeight="1">
-      <c r="A24" s="12" t="inlineStr">
-        <is>
-          <t>Yassine
-contrat 35h</t>
-        </is>
-      </c>
-      <c r="B24" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="C24" s="14" t="inlineStr">
-        <is>
-          <t>09:50 – 14:00
-15:00 – 17:50
-7h00</t>
-        </is>
-      </c>
-      <c r="D24" s="20" t="inlineStr">
-        <is>
-          <t>11:40 – 15:00
-16:00 – 19:40
-7h00</t>
-        </is>
-      </c>
-      <c r="E24" s="18" t="inlineStr">
-        <is>
-          <t>11:00 – 14:00
-15:00 – 19:00
-7h00</t>
-        </is>
-      </c>
-      <c r="F24" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="G24" s="20" t="inlineStr">
-        <is>
-          <t>11:40 – 15:00
-16:00 – 19:40
-7h00</t>
-        </is>
-      </c>
-      <c r="H24" s="26" t="inlineStr">
-        <is>
-          <t>Férié
-non travaillé
-7h00</t>
-        </is>
-      </c>
-      <c r="I24" s="17" t="inlineStr">
-        <is>
-          <t>35h00</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="58" customHeight="1">
-      <c r="A25" s="12" t="inlineStr">
-        <is>
-          <t>Rose
-contrat 35h</t>
-        </is>
-      </c>
-      <c r="B25" s="14" t="inlineStr">
-        <is>
-          <t>09:50 – 14:00
-15:00 – 17:50
-7h00</t>
-        </is>
-      </c>
-      <c r="C25" s="14" t="inlineStr">
-        <is>
-          <t>09:50 – 14:00
-15:00 – 17:50
-7h00</t>
-        </is>
-      </c>
-      <c r="D25" s="14" t="inlineStr">
-        <is>
-          <t>09:50 – 14:00
-15:00 – 17:50
-7h00</t>
-        </is>
-      </c>
-      <c r="E25" s="14" t="inlineStr">
-        <is>
-          <t>09:50 – 14:00
-15:00 – 17:50
-7h00</t>
-        </is>
-      </c>
-      <c r="F25" s="14" t="inlineStr">
-        <is>
-          <t>09:50 – 14:00
-15:00 – 17:50
-7h00</t>
-        </is>
-      </c>
-      <c r="G25" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="H25" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="I25" s="17" t="inlineStr">
-        <is>
-          <t>35h00</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="58" customHeight="1">
-      <c r="A26" s="12" t="inlineStr">
-        <is>
-          <t>Jennyfer
-contrat 25h</t>
-        </is>
-      </c>
-      <c r="B26" s="20" t="inlineStr">
+      <c r="F26" s="20" t="inlineStr">
         <is>
           <t>12:25 – 15:00
 16:00 – 19:40
 6h15</t>
         </is>
       </c>
-      <c r="C26" s="20" t="inlineStr">
-        <is>
-          <t>12:25 – 15:00
-16:00 – 19:40
-6h15</t>
-        </is>
-      </c>
-      <c r="D26" s="19" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="E26" s="20" t="inlineStr">
-        <is>
-          <t>12:25 – 15:00
-16:00 – 19:40
-6h15</t>
-        </is>
-      </c>
-      <c r="F26" s="20" t="inlineStr">
-        <is>
-          <t>12:25 – 15:00
-16:00 – 19:40
-6h15</t>
-        </is>
-      </c>
       <c r="G26" s="15" t="inlineStr">
         <is>
           <t>Congé</t>
@@ -1796,22 +1798,30 @@
     <row r="34" ht="28" customHeight="1">
       <c r="A34" s="28" t="inlineStr">
         <is>
-          <t>• Livraisons : 3 personnes le jeu 15 et le jeu 29 ; 2 personnes les ven 16, jeu 22, ven 23, ven 30.</t>
+          <t>• Semaine du 19/10 : +5h pour Yassine, Rose et Jennyfer (au lieu d'un intérimaire) → Yassine 40h, Rose 40h (part à 18:50), Jennyfer 30h ; 3 personnes les jeu 22 et ven 23 (livraisons).</t>
         </is>
       </c>
     </row>
     <row r="35" ht="28" customHeight="1">
       <c r="A35" s="28" t="inlineStr">
         <is>
+          <t>• Livraisons : 3 personnes les jeu 15, jeu 22, ven 23 et jeu 29 ; 2 personnes les ven 16 et ven 30.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="28" customHeight="1">
+      <c r="A36" s="28" t="inlineStr">
+        <is>
           <t>• Sara indispo sam 24 + dim 25 · Jennyfer en congé du 31/10 au 2/11 · Dim 1/11 (Toussaint) : heures prévues comptées (férié chômé) ; pour Sara (&lt; 3 mois d'ancienneté), paiement à vérifier avec la paie.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A33:I33"/>
     <mergeCell ref="A5:I5"/>
     <mergeCell ref="A32:I32"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A14:I14"/>
     <mergeCell ref="A31:I31"/>
     <mergeCell ref="A22:I22"/>

</xml_diff>